<commit_message>
data: screener 2026-05-27 13:55 IST
</commit_message>
<xml_diff>
--- a/docs/archive/NSE_DMA_Screener_2026-05-27.xlsx
+++ b/docs/archive/NSE_DMA_Screener_2026-05-27.xlsx
@@ -858,7 +858,7 @@
         <v>676749</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1044160</v>
+        <v>952010</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1575.79</v>
+        <v>1578.09</v>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1516.21</v>
+        <v>1517.19</v>
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1411.9</v>
+        <v>1413.02</v>
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="T4" s="2" t="n">
-        <v>40.05</v>
+        <v>39.94</v>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
@@ -14597,7 +14597,7 @@
         <v>676749</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1044160</v>
+        <v>952010</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -14613,7 +14613,7 @@
         </is>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1575.79</v>
+        <v>1578.09</v>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
@@ -14621,7 +14621,7 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1516.21</v>
+        <v>1517.19</v>
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
@@ -14629,7 +14629,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1411.9</v>
+        <v>1413.02</v>
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
@@ -14637,7 +14637,7 @@
         </is>
       </c>
       <c r="T4" s="2" t="n">
-        <v>40.05</v>
+        <v>39.94</v>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>

</xml_diff>